<commit_message>
chore(examples): rename owner workbooks, regenerate template/demo
- Rename pyq.xlsx → richard_network.xlsx and contacts.xlsx →
  tommy_network.xlsx so the example sources match the owner identities
  used by --owner richard / --owner tommy throughout the CLI and UI.
- Regenerate template.xlsx and demo_network.xlsx via the build scripts
  with the new 直接 / 弱认识 / 未联系 vocabulary, updated in-cell
  validations, help text and the "未联系" highlight format.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/examples/demo_network.xlsx
+++ b/examples/demo_network.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="331">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="332">
   <si>
     <t>序号</t>
   </si>
@@ -684,10 +684,10 @@
     <t>高质量项目源; 长期 LP 关系</t>
   </si>
   <si>
-    <t>目标人物 · 圈内可引荐</t>
-  </si>
-  <si>
-    <t>目标</t>
+    <t>想接触 · 圈内可引荐</t>
+  </si>
+  <si>
+    <t>未联系</t>
   </si>
   <si>
     <t>张磊</t>
@@ -915,10 +915,13 @@
     <t>• 没数据的格留空就行，不要填 `-` `无` `NA`。</t>
   </si>
   <si>
-    <t>2. 关键列：关系类型 ⭐ 新增</t>
-  </si>
-  <si>
-    <t>三选一，决定『你』和此人之间是否建立直接好友关系：</t>
+    <t>2. 关键列：关系类型</t>
+  </si>
+  <si>
+    <t>三选一，决定『你』和此人之间是否建立直接好友关系（**不影响搜索本身**——</t>
+  </si>
+  <si>
+    <t>搜索按相关性排序，任何人都可能是你下次自然语言查询的最佳匹配）：</t>
   </si>
   <si>
     <t>• 留空 / 直接 — 默认。把『可信度』作为 Me→此人的边强度。</t>
@@ -927,13 +930,13 @@
     <t>• 弱认识 — 仅强度 1 的边。点头之交、刚加微信、被介绍认识但未深交。</t>
   </si>
   <si>
-    <t>• 目标   — 你不直接认识此人，但希望被引荐到。系统会通过别人的</t>
-  </si>
-  <si>
-    <t xml:space="preserve">          『认识』列推算 2-3 跳的最优引荐路径。Demo 表里</t>
-  </si>
-  <si>
-    <t xml:space="preserve">          沈南鹏/张磊/朱啸虎/雷军/张一鸣/段永平/邱国鹭 都是这种。</t>
+    <t>• 未联系 — 你还没直接联系到此人，但希望被引荐到。系统会通过别人的</t>
+  </si>
+  <si>
+    <t xml:space="preserve">           『认识』列推算 2-3 跳的最优引荐路径。Demo 表里</t>
+  </si>
+  <si>
+    <t xml:space="preserve">           沈南鹏/张磊/朱啸虎/雷军/张一鸣/段永平/邱国鹭 都是这种。</t>
   </si>
   <si>
     <t>3. 关键列：认识</t>
@@ -960,7 +963,7 @@
     <t>• 如果填的人不在表里，导入时会警告并跳过</t>
   </si>
   <si>
-    <t>• ★ 想被引荐到某个『目标』，就在中间人那一行的『认识』里写上目标人物。</t>
+    <t>• ★ 想被引荐到某个『未联系』的人，就在中间人那一行的『认识』里写上他。</t>
   </si>
   <si>
     <t>4. 关键列：公司</t>
@@ -978,7 +981,7 @@
     <t>1-5 分。1 = 认识但不熟；3 = 普通朋友；5 = 核心挚友/铁磁。</t>
   </si>
   <si>
-    <t>对『目标』类型的人填 0 即可（系统忽略）。</t>
+    <t>对『未联系』类型的人填 0 即可（系统忽略）。</t>
   </si>
   <si>
     <t>6. 潜在需求</t>
@@ -3274,7 +3277,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A39"/>
+  <dimension ref="A1:A40"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="110.7109375" customWidth="1"/>
@@ -3340,23 +3343,23 @@
         <v>304</v>
       </c>
     </row>
-    <row r="14" spans="1:1" ht="26" customHeight="1">
-      <c r="A14" s="6" t="s">
+    <row r="14" spans="1:1" ht="22" customHeight="1">
+      <c r="A14" s="7" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="15" spans="1:1" ht="22" customHeight="1">
-      <c r="A15" s="7" t="s">
+    <row r="15" spans="1:1" ht="26" customHeight="1">
+      <c r="A15" s="6" t="s">
         <v>306</v>
       </c>
     </row>
     <row r="16" spans="1:1" ht="22" customHeight="1">
-      <c r="A16" s="8" t="s">
+      <c r="A16" s="7" t="s">
         <v>307</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="22" customHeight="1">
-      <c r="A17" s="7" t="s">
+      <c r="A17" s="8" t="s">
         <v>308</v>
       </c>
     </row>
@@ -3385,13 +3388,13 @@
         <v>313</v>
       </c>
     </row>
-    <row r="23" spans="1:1" ht="26" customHeight="1">
-      <c r="A23" s="6" t="s">
+    <row r="23" spans="1:1" ht="22" customHeight="1">
+      <c r="A23" s="7" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="24" spans="1:1" ht="22" customHeight="1">
-      <c r="A24" s="7" t="s">
+    <row r="24" spans="1:1" ht="26" customHeight="1">
+      <c r="A24" s="6" t="s">
         <v>315</v>
       </c>
     </row>
@@ -3400,13 +3403,13 @@
         <v>316</v>
       </c>
     </row>
-    <row r="26" spans="1:1" ht="26" customHeight="1">
-      <c r="A26" s="6" t="s">
+    <row r="26" spans="1:1" ht="22" customHeight="1">
+      <c r="A26" s="7" t="s">
         <v>317</v>
       </c>
     </row>
-    <row r="27" spans="1:1" ht="22" customHeight="1">
-      <c r="A27" s="7" t="s">
+    <row r="27" spans="1:1" ht="26" customHeight="1">
+      <c r="A27" s="6" t="s">
         <v>318</v>
       </c>
     </row>
@@ -3415,13 +3418,13 @@
         <v>319</v>
       </c>
     </row>
-    <row r="29" spans="1:1" ht="26" customHeight="1">
-      <c r="A29" s="6" t="s">
+    <row r="29" spans="1:1" ht="22" customHeight="1">
+      <c r="A29" s="7" t="s">
         <v>320</v>
       </c>
     </row>
-    <row r="30" spans="1:1" ht="22" customHeight="1">
-      <c r="A30" s="7" t="s">
+    <row r="30" spans="1:1" ht="26" customHeight="1">
+      <c r="A30" s="6" t="s">
         <v>321</v>
       </c>
     </row>
@@ -3430,13 +3433,13 @@
         <v>322</v>
       </c>
     </row>
-    <row r="32" spans="1:1" ht="26" customHeight="1">
-      <c r="A32" s="6" t="s">
+    <row r="32" spans="1:1" ht="22" customHeight="1">
+      <c r="A32" s="7" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="33" spans="1:1" ht="22" customHeight="1">
-      <c r="A33" s="7" t="s">
+    <row r="33" spans="1:1" ht="26" customHeight="1">
+      <c r="A33" s="6" t="s">
         <v>324</v>
       </c>
     </row>
@@ -3450,24 +3453,29 @@
         <v>326</v>
       </c>
     </row>
-    <row r="36" spans="1:1" ht="26" customHeight="1">
-      <c r="A36" s="6" t="s">
+    <row r="36" spans="1:1" ht="22" customHeight="1">
+      <c r="A36" s="7" t="s">
         <v>327</v>
       </c>
     </row>
-    <row r="37" spans="1:1" ht="22" customHeight="1">
-      <c r="A37" s="7" t="s">
+    <row r="37" spans="1:1" ht="26" customHeight="1">
+      <c r="A37" s="6" t="s">
         <v>328</v>
       </c>
     </row>
     <row r="38" spans="1:1" ht="22" customHeight="1">
-      <c r="A38" s="8" t="s">
+      <c r="A38" s="7" t="s">
         <v>329</v>
       </c>
     </row>
     <row r="39" spans="1:1" ht="22" customHeight="1">
-      <c r="A39" s="7" t="s">
+      <c r="A39" s="8" t="s">
         <v>330</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" ht="22" customHeight="1">
+      <c r="A40" s="7" t="s">
+        <v>331</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: collapse 关系类型 to binary 已联系/未联系
把"关系类型"档位从三态（直接/弱认识/未联系）收成二态（已联系/未联系）。
旧版本的"弱认识"档位本质上是 strength=1 的快捷方式，与"可信度 1-5"列
重复表达"有多熟"这一语义。彻底废弃后，三个维度终于正交：

  - 事实：是否联系到 → kind_column ∈ {已联系, 未联系}
  - 强度：联系到的有多熟 → 可信度 1-5（1 即点头之交）
  - 意图：下次想找谁 → web 端搜索框那句自然语言（LLM 解析，不入库）

填表人不再需要在表里预先标"谁是想接触的目标"——任何人都可能成为某次
查询的最佳匹配，搜索按相关性排序。

importer:
  - 删 _KIND_DIRECT / _KIND_WEAK 常量与 strength=1 强制路径
  - _normalize_kind 仅识别 已联系/contacted/留空 vs 未联系/uncontacted
  - 旧词（直接/弱认识/目标/想认识/target/陌生）silent fallback 到默认
    已联系，按可信度建 Me 边

template / demo:
  - data_validation 下拉收成二选一
  - 删 fmt_weak 配色，sample 行更新为 已联系×2 / 未联系×1
  - 「说明」sheet 与列描述强调"事实 vs 意图"边界

frontend:
  - 删 weak 段落，与 direct 合并为单段「你已联系的人」，按 combined_score
    排序（strength=1 自然落到段末）
  - summary chip 收成 "N 已联系 · M 需引荐"

docs:
  - network_template_guide / instructions / progress-report 同步收成二态
  - 重申"关系类型只描述事实，不要在表里预定义谁是目标"

tests: - test_kind_legacy_values_collapse_to_contacted: 锁住"弱认识"不再走
    strength=1 捷径，必须按可信度落地
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/examples/demo_network.xlsx
+++ b/examples/demo_network.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="332">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="334">
   <si>
     <t>序号</t>
   </si>
@@ -915,25 +915,31 @@
     <t>• 没数据的格留空就行，不要填 `-` `无` `NA`。</t>
   </si>
   <si>
-    <t>2. 关键列：关系类型</t>
-  </si>
-  <si>
-    <t>三选一，决定『你』和此人之间是否建立直接好友关系（**不影响搜索本身**——</t>
+    <t>2. 关键列：关系类型（二态、纯事实）</t>
+  </si>
+  <si>
+    <t>二选一，只描述『我和此人有没有联系上』，**不描述意图**。</t>
+  </si>
+  <si>
+    <t>（『下次想找谁』是 web 端搜索框里那句自然语言决定的，不要在表里预定义谁是『目标』。）</t>
+  </si>
+  <si>
+    <t>**不影响搜索本身**——</t>
   </si>
   <si>
     <t>搜索按相关性排序，任何人都可能是你下次自然语言查询的最佳匹配）：</t>
   </si>
   <si>
-    <t>• 留空 / 直接 — 默认。把『可信度』作为 Me→此人的边强度。</t>
-  </si>
-  <si>
-    <t>• 弱认识 — 仅强度 1 的边。点头之交、刚加微信、被介绍认识但未深交。</t>
-  </si>
-  <si>
-    <t>• 未联系 — 你还没直接联系到此人，但希望被引荐到。系统会通过别人的</t>
-  </si>
-  <si>
-    <t xml:space="preserve">           『认识』列推算 2-3 跳的最优引荐路径。Demo 表里</t>
+    <t>• 留空 / 已联系 — 默认。把『可信度』作为 Me→此人的边强度（1-5，</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                  1 = 点头之交，5 = 核心铁磁）。</t>
+  </si>
+  <si>
+    <t>• 未联系 — 我还没直接联系到此人。系统会通过别人的『认识』列推算</t>
+  </si>
+  <si>
+    <t xml:space="preserve">           2-3 跳的最优引荐路径。Demo 表里</t>
   </si>
   <si>
     <t xml:space="preserve">           沈南鹏/张磊/朱啸虎/雷军/张一鸣/段永平/邱国鹭 都是这种。</t>
@@ -3277,7 +3283,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A40"/>
+  <dimension ref="A1:A42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="110.7109375" customWidth="1"/>
@@ -3348,8 +3354,8 @@
         <v>305</v>
       </c>
     </row>
-    <row r="15" spans="1:1" ht="26" customHeight="1">
-      <c r="A15" s="6" t="s">
+    <row r="15" spans="1:1" ht="22" customHeight="1">
+      <c r="A15" s="7" t="s">
         <v>306</v>
       </c>
     </row>
@@ -3358,8 +3364,8 @@
         <v>307</v>
       </c>
     </row>
-    <row r="17" spans="1:1" ht="22" customHeight="1">
-      <c r="A17" s="8" t="s">
+    <row r="17" spans="1:1" ht="26" customHeight="1">
+      <c r="A17" s="6" t="s">
         <v>308</v>
       </c>
     </row>
@@ -3369,7 +3375,7 @@
       </c>
     </row>
     <row r="19" spans="1:1" ht="22" customHeight="1">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="8" t="s">
         <v>310</v>
       </c>
     </row>
@@ -3393,8 +3399,8 @@
         <v>314</v>
       </c>
     </row>
-    <row r="24" spans="1:1" ht="26" customHeight="1">
-      <c r="A24" s="6" t="s">
+    <row r="24" spans="1:1" ht="22" customHeight="1">
+      <c r="A24" s="7" t="s">
         <v>315</v>
       </c>
     </row>
@@ -3403,13 +3409,13 @@
         <v>316</v>
       </c>
     </row>
-    <row r="26" spans="1:1" ht="22" customHeight="1">
-      <c r="A26" s="7" t="s">
+    <row r="26" spans="1:1" ht="26" customHeight="1">
+      <c r="A26" s="6" t="s">
         <v>317</v>
       </c>
     </row>
-    <row r="27" spans="1:1" ht="26" customHeight="1">
-      <c r="A27" s="6" t="s">
+    <row r="27" spans="1:1" ht="22" customHeight="1">
+      <c r="A27" s="7" t="s">
         <v>318</v>
       </c>
     </row>
@@ -3418,13 +3424,13 @@
         <v>319</v>
       </c>
     </row>
-    <row r="29" spans="1:1" ht="22" customHeight="1">
-      <c r="A29" s="7" t="s">
+    <row r="29" spans="1:1" ht="26" customHeight="1">
+      <c r="A29" s="6" t="s">
         <v>320</v>
       </c>
     </row>
-    <row r="30" spans="1:1" ht="26" customHeight="1">
-      <c r="A30" s="6" t="s">
+    <row r="30" spans="1:1" ht="22" customHeight="1">
+      <c r="A30" s="7" t="s">
         <v>321</v>
       </c>
     </row>
@@ -3433,13 +3439,13 @@
         <v>322</v>
       </c>
     </row>
-    <row r="32" spans="1:1" ht="22" customHeight="1">
-      <c r="A32" s="7" t="s">
+    <row r="32" spans="1:1" ht="26" customHeight="1">
+      <c r="A32" s="6" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="33" spans="1:1" ht="26" customHeight="1">
-      <c r="A33" s="6" t="s">
+    <row r="33" spans="1:1" ht="22" customHeight="1">
+      <c r="A33" s="7" t="s">
         <v>324</v>
       </c>
     </row>
@@ -3448,8 +3454,8 @@
         <v>325</v>
       </c>
     </row>
-    <row r="35" spans="1:1" ht="22" customHeight="1">
-      <c r="A35" s="7" t="s">
+    <row r="35" spans="1:1" ht="26" customHeight="1">
+      <c r="A35" s="6" t="s">
         <v>326</v>
       </c>
     </row>
@@ -3458,8 +3464,8 @@
         <v>327</v>
       </c>
     </row>
-    <row r="37" spans="1:1" ht="26" customHeight="1">
-      <c r="A37" s="6" t="s">
+    <row r="37" spans="1:1" ht="22" customHeight="1">
+      <c r="A37" s="7" t="s">
         <v>328</v>
       </c>
     </row>
@@ -3468,14 +3474,24 @@
         <v>329</v>
       </c>
     </row>
-    <row r="39" spans="1:1" ht="22" customHeight="1">
-      <c r="A39" s="8" t="s">
+    <row r="39" spans="1:1" ht="26" customHeight="1">
+      <c r="A39" s="6" t="s">
         <v>330</v>
       </c>
     </row>
     <row r="40" spans="1:1" ht="22" customHeight="1">
       <c r="A40" s="7" t="s">
         <v>331</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" ht="22" customHeight="1">
+      <c r="A41" s="8" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" ht="22" customHeight="1">
+      <c r="A42" s="7" t="s">
+        <v>333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>